<commit_message>
client: rút nhãn màn thăng tinh cho khỏi đè số ("Cấp tối đa:", "Công/máu:", "Tốc độ:")
Ô nhãn trong box1Lv/box1Desc1 rộng 130px chữ 24px, giá trị đứng ở x=152; nhãn dịch máy
21–22 ký tự ("Cấp hạn mức cao nhất:", "Công máu trưởng thành:") đè lên "255 » 280". Thêm ba
quy tắc vào bảng thuật ngữ — riêng "tốc độ tăng lên" chỉ khớp dạng nhãn có dấu hai chấm, vì
cụm không dấu chấm xuất hiện 522 lần trong mô tả kỹ năng/buff ("tốc độ tăng lên 10%").
ui.bin -> res/aace3-6ad1f-baa8e, templates.bin -> res/97cec-435a4-5f56f (đã chép assets +
docker cp manifest); 3 workbook máy chủ biên dịch lại, ExcelProbe OK.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/excel/release/system-prompt-localization.xlsx
+++ b/server/excel/release/system-prompt-localization.xlsx
@@ -2310,13 +2310,13 @@
     <t xml:space="preserve">速度提升:</t>
   </si>
   <si>
-    <t xml:space="preserve">Tốc độ tăng lên:</t>
+    <t xml:space="preserve">Tốc độ:</t>
   </si>
   <si>
     <t xml:space="preserve">攻血成长:</t>
   </si>
   <si>
-    <t xml:space="preserve">Công máu trưởng thành:</t>
+    <t xml:space="preserve">Công/máu:</t>
   </si>
   <si>
     <t xml:space="preserve">攻击成长:</t>

</xml_diff>